<commit_message>
Wire month-start AR baseline file and UR tracking consolidation into the weekly deck
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_01GRGYp2p9fdXmxQMcLgyM1e
</commit_message>
<xml_diff>
--- a/weekly-ar-cash-deck/inputs/weekly_inputs.xlsx
+++ b/weekly-ar-cash-deck/inputs/weekly_inputs.xlsx
@@ -17,18 +17,20 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AR_UNPAID_STATUS" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AR_AGING" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UNRECOGNIZED" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COLLECTIONS_BU" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COLLECTIONS_MONTHLY" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH_MONTHLY" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH_BU" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH_BU_OCT" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ONGOING" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_BU" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_BUCKETS" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_BU_ORIGIN" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_TIERS" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_TOP_SUPPLIERS" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LC_LINES" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UR_ATTACHMENT_STATUS" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UR_PO_SUMMARY" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COLLECTIONS_BU" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COLLECTIONS_MONTHLY" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH_MONTHLY" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH_BU" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH_BU_OCT" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ONGOING" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_BU" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_BUCKETS" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_BU_ORIGIN" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_TIERS" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP_TOP_SUPPLIERS" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LC_LINES" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -545,7 +547,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -644,7 +646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -661,12 +663,13 @@
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Unrecognized suppliers (equipment + subcontracts) by status, MMAD, current week.</t>
+          <t>Unrecognized suppliers (equipment + subcontracts) by status, MMAD incl. markup, current week; prev_week_total = previous BU update (incl. markup).</t>
         </is>
       </c>
     </row>
@@ -741,6 +744,11 @@
           <t>grand_total</t>
         </is>
       </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>prev_week_total</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -787,6 +795,9 @@
       <c r="N3" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="O3" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -795,13 +806,13 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>74.74699200000001</v>
+        <v>80.06459096406002</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>3.776969</v>
+        <v>3.77696858</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>0.856001</v>
+        <v>0.8560008193</v>
       </c>
       <c r="E4" s="4" t="n">
         <v>0</v>
@@ -810,28 +821,31 @@
         <v>0</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>36.637994</v>
+        <v>36.63799390625</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>4.609417</v>
+        <v>4.6094170221</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>3.748898</v>
+        <v>3.748897873599999</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>2.609802</v>
+        <v>2.60980175775</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>126.986073</v>
+        <v>132.30367092306</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>0.190829</v>
+        <v>0.19082879</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>127.176902</v>
+        <v>132.49449971306</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>58.541424083405</v>
       </c>
     </row>
     <row r="5">
@@ -879,6 +893,9 @@
       <c r="N5" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="O5" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -887,13 +904,13 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>0.7411990000000001</v>
+        <v>0.6837</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>0.747644</v>
+        <v>0.3657</v>
       </c>
       <c r="E6" s="4" t="n">
         <v>0</v>
@@ -902,28 +919,31 @@
         <v>0</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>43.655921</v>
+        <v>47.6371975228</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1.250958</v>
+        <v>1.9240583534</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>0.369135</v>
+        <v>1.2527904044</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>6.34835</v>
+        <v>6.34834954</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>53.113207</v>
+        <v>58.2117958206</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>0.059072</v>
+        <v>0.05907168</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>53.172279</v>
+        <v>58.2708675006</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>95.15545376</v>
       </c>
     </row>
     <row r="7">
@@ -948,10 +968,10 @@
         <v>0</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>30.476683</v>
+        <v>30.47668346019995</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>331.199265</v>
+        <v>331.1992646145408</v>
       </c>
       <c r="I7" s="4" t="n">
         <v>0</v>
@@ -963,13 +983,16 @@
         <v>0</v>
       </c>
       <c r="L7" s="4" t="n">
-        <v>361.675948</v>
+        <v>361.6759480747407</v>
       </c>
       <c r="M7" s="4" t="n">
         <v>0</v>
       </c>
       <c r="N7" s="4" t="n">
-        <v>361.675948</v>
+        <v>361.6759480747407</v>
+      </c>
+      <c r="O7" s="4" t="n">
+        <v>113.572382579</v>
       </c>
     </row>
     <row r="8">
@@ -979,43 +1002,46 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>68.092782</v>
+        <v>72.73827371406801</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>20.796185</v>
+        <v>19.83686351504001</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>120.838124</v>
+        <v>112.2987610638308</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>173.510833</v>
+        <v>173.4470195117179</v>
       </c>
       <c r="F8" s="4" t="n">
         <v>0</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>295.765179</v>
+        <v>295.7651792116337</v>
       </c>
       <c r="H8" s="4" t="n">
         <v>0</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>370.880931</v>
+        <v>370.880930673184</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>310.105385</v>
+        <v>310.1053847773999</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>1.658972</v>
+        <v>1.6589716772</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>1361.648391</v>
+        <v>1356.731384144074</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>24.937958</v>
+        <v>24.9379583268</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>1386.586349</v>
+        <v>1381.669342470875</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>1539.001549975228</v>
       </c>
     </row>
     <row r="9">
@@ -1025,43 +1051,46 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>5.922738</v>
+        <v>5.922737598</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>4.952486</v>
+        <v>4.952486432720001</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>10.689496</v>
+        <v>10.6894961392</v>
       </c>
       <c r="F9" s="4" t="n">
         <v>0</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>35.121441</v>
+        <v>41.98374752234158</v>
       </c>
       <c r="H9" s="4" t="n">
         <v>0</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>26.38352</v>
+        <v>14.6547596152</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>138.717595</v>
+        <v>75.91532683982847</v>
       </c>
       <c r="K9" s="4" t="n">
-        <v>3.389336</v>
+        <v>3.389335531</v>
       </c>
       <c r="L9" s="4" t="n">
-        <v>225.176612</v>
+        <v>157.50788967829</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>2.743711</v>
+        <v>2.7437112716</v>
       </c>
       <c r="N9" s="4" t="n">
-        <v>227.920323</v>
+        <v>160.25160094989</v>
+      </c>
+      <c r="O9" s="4" t="n">
+        <v>347.1237891044</v>
       </c>
     </row>
     <row r="10">
@@ -1077,7 +1106,7 @@
         <v>0</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>249.490044</v>
+        <v>249.490043642212</v>
       </c>
       <c r="E10" s="4" t="n">
         <v>0</v>
@@ -1101,13 +1130,16 @@
         <v>0</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>252.212124</v>
+        <v>252.212123642212</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>0</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>252.212124</v>
+        <v>252.212123642212</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>438.1603746820252</v>
       </c>
     </row>
     <row r="11">
@@ -1117,28 +1149,28 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>43.259442</v>
+        <v>47.56506507399999</v>
       </c>
       <c r="C11" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>911.153867</v>
+        <v>1060.5555333754</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>179.159034</v>
+        <v>291.401692208</v>
       </c>
       <c r="F11" s="4" t="n">
         <v>0</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>266.469767</v>
+        <v>174.9286514714</v>
       </c>
       <c r="H11" s="4" t="n">
         <v>0</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>918.822728</v>
+        <v>1696.174394165814</v>
       </c>
       <c r="J11" s="4" t="n">
         <v>0</v>
@@ -1147,13 +1179,16 @@
         <v>0</v>
       </c>
       <c r="L11" s="4" t="n">
-        <v>2318.864838</v>
+        <v>3270.625336294613</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>1351.539037</v>
+        <v>0</v>
       </c>
       <c r="N11" s="4" t="n">
-        <v>3670.403875</v>
+        <v>3270.625336294613</v>
+      </c>
+      <c r="O11" s="4" t="n">
+        <v>3466.546150650921</v>
       </c>
     </row>
     <row r="12">
@@ -1163,43 +1198,46 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>49.90055</v>
+        <v>49.880438083706</v>
       </c>
       <c r="C12" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>95.931934</v>
+        <v>95.93193427602603</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>22.179109</v>
+        <v>22.179109313284</v>
       </c>
       <c r="F12" s="4" t="n">
         <v>0</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>333.831796</v>
+        <v>333.8330972426266</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>1.610311</v>
+        <v>0.2167176</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>150.010502</v>
+        <v>149.9988008924615</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>859.089018</v>
+        <v>859.0890177651654</v>
       </c>
       <c r="K12" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>1512.55322</v>
+        <v>1511.12911517327</v>
       </c>
       <c r="M12" s="4" t="n">
         <v>0</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>1512.55322</v>
+        <v>1511.12911517327</v>
+      </c>
+      <c r="O12" s="4" t="n">
+        <v>1735.797329236808</v>
       </c>
     </row>
   </sheetData>
@@ -1208,6 +1246,748 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Status of JESA attachments to client (UR consolidation, MMAD incl. markup).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>bu</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>eq_under_jesa_approval</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>eq_under_jesa_preparation</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>eq_under_client_approval</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>eq_signed_by_client</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>eq_accrual_posted</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>sub_under_jesa_approval</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>sub_under_jesa_preparation</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>sub_under_client_approval</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>sub_signed_by_client</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>sub_accrual_posted</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Advisory</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>73.19426740011002</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>6.870323563949999</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>3.77696858</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>32.7983390262</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>1.32974597855</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>2.5099089015</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>4.6094170221</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>125.08897047241</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Capabilities</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>0.6837</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>42.9828207222</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>0.03869000000000047</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>4.615686800599998</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>1.9240583534</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>50.2449558762</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Energy Operations</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>4.375793017199993</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>26.10089044299996</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>331.1992646145408</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="4" t="n">
+        <v>361.6759480747407</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Fertilizers &amp; Chemicals</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>19.74332273596001</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>41.01577216270801</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>11.9791788154</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>19.83686351504001</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>295.5038196968337</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>0.2613595148</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>0.3552696</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>388.6955860407417</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Global Mining</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>5.922737598</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>23.63470670014159</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>18.3490408222</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>3.199972202000001</v>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="4" t="n">
+        <v>51.10645732234158</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>JESA Technologies</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>2.72208</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>2.72208</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>SP2M Ad Hoc Program</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>0.1435726539999992</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>35.67199449999998</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>11.74949792</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>174.9286514714</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="4" t="n">
+        <v>222.4937165454</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Water &amp; Environment</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>49.79484212970601</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>0.08559595400000002</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>332.35569399876</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>0.001301441666666535</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>1.4761018022</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>0.3117996</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>384.0253349263327</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Supplier PO consolidation by BU (MMAD): contract value, recognized (SAP GR), unrecognized, remaining.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>bu</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>contract_value</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>recognized</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>unrecognized</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>remaining</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Advisory</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>SP2M Ad Hoc Program</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>10176.53929093992</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>3738.803935507842</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>2036.353988603164</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>4401.381366828909</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>220.4752240775291</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>132.578999179533</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>119.0203539579999</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>-31.124129060004</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Fertilizers &amp; Chemicals</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>3056.338487099643</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>1442.850666636691</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>981.9266487278809</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>631.5611717350732</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Capabilities</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Energy Operations</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>1173.26571524</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>431.86252457</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>341.203724598812</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>400.199466071188</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Building &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>120.6393464257</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>58.863696882522</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>48.85019100999999</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>12.92545853317799</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>JESA Technologies</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>578.1806385486</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>337.351223912097</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>237.9359657002</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>2.893448936302975</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Global Mining</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>789.0336393234729</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>285.979424674361</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>102.8427052770015</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>400.2115093721105</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Water &amp; Environment</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>5716.718243207954</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>4265.655652009003</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>616.610123136089</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>834.4524680628651</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1549,7 +2329,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1748,7 +2528,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2115,7 +2895,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2540,7 +3320,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2857,7 +3637,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3116,7 +3896,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3505,7 +4285,125 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="120" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Auto-drafted from the numbers; rewrite the wording as needed (max 5 messages).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>body</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total AR down 162 MMAD vs last week and down 164 MMAD vs the month-start (07 Oct) baseline</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Total AR stands at 12,689 MMAD (−162 WoW, −164 vs month start). Adding 7,128 MMAD of unrecognized revenue (−666 vs the previous BU update), gross exposure is 19,817 MMAD. Unbilled is 9,514 MMAD (75% of AR, −168 WoW); unpaid is 2,627 MMAD (+6 WoW, +6 vs baseline).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Collections: 110 MMAD received in October to date (+82 WoW), 7,357 MMAD YTD</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>October receipts moved from 27 to 110 MMAD this week. YTD payments received reach 7,357 MMAD (7.36 Bn MAD).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Procurement cash position: net −171 MMAD Jul–Oct including October commitments</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Cumulative procurement cash IN of 2,104 MMAD vs cash OUT of 2,276 MMAD (Jul–Sep actuals, Oct actuals to 15/10, plus 321 MMAD of approved and pending October commitments). October alone: 151 MMAD in vs 220 MMAD paid, 321 MMAD still to pay.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Payables: 2,144 MMAD of supplier invoices in AP (4411 + parked + downpayments), 1,415 MMAD past due</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>2,803 open supplier lines. Parked invoices and 4411 open items dominate; see the AP slide for due-date buckets, tiers and top suppliers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Letters of credit: 912 MMAD outstanding on opened LCs, 1,583 MMAD including LCs still to be opened</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>October LC maturities of 156 MMAD are counted as approved payments in the cash position. 675 MMAD falls in 2026 and 908 MMAD in 2027 per the maturity schedule.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3713,7 +4611,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4176,125 +5074,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
-    <col width="120" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Auto-drafted from the numbers; rewrite the wording as needed (max 5 messages).</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>body</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Total AR down 162 MMAD vs last week and down 551 MMAD vs the 01 Aug baseline</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Total AR stands at 12,689 MMAD (−162 WoW, −551 vs baseline). Adding 7,592 MMAD of unrecognized revenue, gross exposure is 20,281 MMAD. Unbilled is 9,514 MMAD (75% of AR, −168 WoW); unpaid is 2,627 MMAD (+6 WoW, −764 vs baseline).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Collections: 110 MMAD received in October to date (+82 WoW), 7,357 MMAD YTD</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>October receipts moved from 27 to 110 MMAD this week. YTD payments received reach 7,357 MMAD (7.36 Bn MAD).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Procurement cash position: net -171 MMAD Jul–Oct including October commitments</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Cumulative procurement cash IN of 2,104 MMAD vs cash OUT of 2,276 MMAD (Jul–Sep actuals, Oct actuals to 15/10, plus 321 MMAD of approved and pending October commitments). October alone: 151 MMAD in vs 220 MMAD paid, 321 MMAD still to pay.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Payables: 2,144 MMAD of supplier invoices in AP (4411 + parked + downpayments), 1,415 MMAD past due</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>2,803 open supplier lines. Parked invoices and 4411 open items dominate; see the AP slide for due-date buckets, tiers and top suppliers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Letters of credit: 912 MMAD outstanding on opened LCs, 1,583 MMAD including LCs still to be opened</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>October LC maturities of 156 MMAD are counted as approved payments in the cash position. 675 MMAD falls in 2026 and 908 MMAD in 2027 per the maturity schedule.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4431,7 +5211,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4699,7 +5479,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11384,7 +12164,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>503.290157936</v>
+        <v>547.4616826512201</v>
       </c>
       <c r="C3" s="4" t="n">
         <v>547.4616826512199</v>
@@ -11400,7 +12180,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>9345.099074795013</v>
+        <v>9683.62880464431</v>
       </c>
       <c r="C4" s="4" t="n">
         <v>9681.98338223435</v>
@@ -11416,7 +12196,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>3391.355713094379</v>
+        <v>2621.817790321611</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>2621.81779032161</v>
@@ -11432,7 +12212,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>13239.74494582539</v>
+        <v>12852.90827761714</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>12851.2628552072</v>
@@ -11451,10 +12231,10 @@
         <v>0</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>7551.891574</v>
+        <v>7793.898454071787</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>7591.70102</v>
+        <v>7128.328833819261</v>
       </c>
     </row>
     <row r="8">
@@ -11467,10 +12247,10 @@
         <v>0</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>7551.891574</v>
+        <v>7793.898454071787</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>7591.70102</v>
+        <v>7128.328833819261</v>
       </c>
     </row>
     <row r="9">
@@ -11483,10 +12263,10 @@
         <v>0</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>20403.1544292072</v>
+        <v>20645.16130927898</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>20280.67767804529</v>
+        <v>19817.30549186455</v>
       </c>
     </row>
     <row r="10">
@@ -11753,7 +12533,7 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>364.4384869319999</v>
+        <v>405.39468494</v>
       </c>
       <c r="D3" s="4" t="n">
         <v>405.39468494</v>
@@ -11774,7 +12554,7 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>2413.852646288111</v>
+        <v>2611.140868802155</v>
       </c>
       <c r="D4" s="4" t="n">
         <v>2611.14086880215</v>
@@ -11795,7 +12575,7 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>1299.871207797087</v>
+        <v>514.8522276229667</v>
       </c>
       <c r="D5" s="4" t="n">
         <v>514.852227622967</v>
@@ -11816,7 +12596,7 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>4078.162341017198</v>
+        <v>3531.387781365122</v>
       </c>
       <c r="D6" s="4" t="n">
         <v>3531.38778136512</v>
@@ -11837,7 +12617,7 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>27.3586558</v>
+        <v>27.2332702</v>
       </c>
       <c r="D7" s="4" t="n">
         <v>27.2332702</v>
@@ -11858,7 +12638,7 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>2556.652375826921</v>
+        <v>2580.142681887315</v>
       </c>
       <c r="D8" s="4" t="n">
         <v>2580.14268188732</v>
@@ -11879,7 +12659,7 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>612.5060329914982</v>
+        <v>626.8968077662972</v>
       </c>
       <c r="D9" s="4" t="n">
         <v>626.896807766298</v>
@@ -11900,7 +12680,7 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>3196.51706461842</v>
+        <v>3234.272759853613</v>
       </c>
       <c r="D10" s="4" t="n">
         <v>3234.27275985362</v>
@@ -11921,7 +12701,7 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>70.36990110000001</v>
+        <v>70.36990109999999</v>
       </c>
       <c r="D11" s="4" t="n">
         <v>70.36990109999999</v>
@@ -11942,7 +12722,7 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>2427.948264599826</v>
+        <v>2812.435181132908</v>
       </c>
       <c r="D12" s="4" t="n">
         <v>2812.43518113291</v>
@@ -11963,7 +12743,7 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>622.4226311220258</v>
+        <v>445.4692008100001</v>
       </c>
       <c r="D13" s="4" t="n">
         <v>445.46920081</v>
@@ -11984,7 +12764,7 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>3120.740796821852</v>
+        <v>3328.274283042908</v>
       </c>
       <c r="D14" s="4" t="n">
         <v>3328.27428304291</v>
@@ -12026,7 +12806,7 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>802.8399841058896</v>
+        <v>685.54455151329</v>
       </c>
       <c r="D16" s="4" t="n">
         <v>685.54455151329</v>
@@ -12047,7 +12827,7 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>215.1476796019999</v>
+        <v>334.5037520650001</v>
       </c>
       <c r="D17" s="4" t="n">
         <v>334.503752065</v>
@@ -12068,7 +12848,7 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>1017.98766370789</v>
+        <v>1020.04830357829</v>
       </c>
       <c r="D18" s="4" t="n">
         <v>1020.04830357829</v>
@@ -12089,7 +12869,7 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>41.123114104</v>
+        <v>40.707594104</v>
       </c>
       <c r="D19" s="4" t="n">
         <v>40.707594104</v>
@@ -12110,7 +12890,7 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>413.4471015600006</v>
+        <v>365.8943560853061</v>
       </c>
       <c r="D20" s="4" t="n">
         <v>365.894356085306</v>
@@ -12131,7 +12911,7 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>128.695441113978</v>
+        <v>92.9369876961136</v>
       </c>
       <c r="D21" s="4" t="n">
         <v>92.9369876961136</v>
@@ -12152,7 +12932,7 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>583.2656567779786</v>
+        <v>499.5389378854197</v>
       </c>
       <c r="D22" s="4" t="n">
         <v>499.53893788542</v>
@@ -12194,7 +12974,7 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>430.8182500924902</v>
+        <v>421.1324197048001</v>
       </c>
       <c r="D24" s="4" t="n">
         <v>421.1324197048</v>
@@ -12215,7 +12995,7 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>108.2669275443064</v>
+        <v>135.9767291956514</v>
       </c>
       <c r="D25" s="4" t="n">
         <v>135.976729195651</v>
@@ -12236,7 +13016,7 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>539.0851776367966</v>
+        <v>557.1091489004515</v>
       </c>
       <c r="D26" s="4" t="n">
         <v>557.1091489004521</v>
@@ -12278,7 +13058,7 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>104.6003067500001</v>
+        <v>147.4579813800002</v>
       </c>
       <c r="D28" s="4" t="n">
         <v>145.81255897</v>
@@ -12299,7 +13079,7 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>339.7218147904763</v>
+        <v>339.5929317804761</v>
       </c>
       <c r="D29" s="4" t="n">
         <v>339.592931780476</v>
@@ -12320,7 +13100,7 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>444.3221215404764</v>
+        <v>487.0509131604763</v>
       </c>
       <c r="D30" s="4" t="n">
         <v>485.405490750476</v>
@@ -12341,7 +13121,7 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>0</v>
+        <v>3.756232307219999</v>
       </c>
       <c r="D31" s="4" t="n">
         <v>3.75623230722</v>
@@ -12362,7 +13142,7 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>144.6670841567733</v>
+        <v>8.364731263063474</v>
       </c>
       <c r="D32" s="4" t="n">
         <v>8.364731263063479</v>
@@ -12383,7 +13163,7 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>34.23922855320699</v>
+        <v>102.725108383306</v>
       </c>
       <c r="D33" s="4" t="n">
         <v>102.725108383306</v>
@@ -12404,7 +13184,7 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>178.9063127099803</v>
+        <v>114.8460719535895</v>
       </c>
       <c r="D34" s="4" t="n">
         <v>114.846071953589</v>
@@ -12446,7 +13226,7 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>45.62995834500001</v>
+        <v>45.53225954550001</v>
       </c>
       <c r="D36" s="4" t="n">
         <v>45.5322595455</v>
@@ -12467,7 +13247,7 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>29.0614083398</v>
+        <v>27.4407037618</v>
       </c>
       <c r="D37" s="4" t="n">
         <v>27.4407037618</v>
@@ -12488,7 +13268,7 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>74.6913666848</v>
+        <v>72.97296330730001</v>
       </c>
       <c r="D38" s="4" t="n">
         <v>72.97296330730001</v>
@@ -12530,7 +13310,7 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>4.643103070000001</v>
+        <v>5.983773330000001</v>
       </c>
       <c r="D40" s="4" t="n">
         <v>5.98377333</v>
@@ -12572,7 +13352,7 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>6.066444310000001</v>
+        <v>7.407114570000001</v>
       </c>
       <c r="D42" s="4" t="n">
         <v>7.40711457</v>
@@ -12612,7 +13392,7 @@
       <c r="C44" s="3" t="n"/>
       <c r="D44" s="3" t="n"/>
       <c r="E44" s="4" t="n">
-        <v>127.176902</v>
+        <v>132.49449971306</v>
       </c>
     </row>
     <row r="45">
@@ -12646,7 +13426,7 @@
       <c r="C46" s="3" t="n"/>
       <c r="D46" s="3" t="n"/>
       <c r="E46" s="4" t="n">
-        <v>53.172279</v>
+        <v>58.2708675006</v>
       </c>
     </row>
     <row r="47">
@@ -12663,7 +13443,7 @@
       <c r="C47" s="3" t="n"/>
       <c r="D47" s="3" t="n"/>
       <c r="E47" s="4" t="n">
-        <v>361.675948</v>
+        <v>361.6759480747407</v>
       </c>
     </row>
     <row r="48">
@@ -12680,7 +13460,7 @@
       <c r="C48" s="3" t="n"/>
       <c r="D48" s="3" t="n"/>
       <c r="E48" s="4" t="n">
-        <v>1386.586349</v>
+        <v>1381.669342470875</v>
       </c>
     </row>
     <row r="49">
@@ -12697,7 +13477,7 @@
       <c r="C49" s="3" t="n"/>
       <c r="D49" s="3" t="n"/>
       <c r="E49" s="4" t="n">
-        <v>227.920323</v>
+        <v>160.25160094989</v>
       </c>
     </row>
     <row r="50">
@@ -12714,7 +13494,7 @@
       <c r="C50" s="3" t="n"/>
       <c r="D50" s="3" t="n"/>
       <c r="E50" s="4" t="n">
-        <v>252.212124</v>
+        <v>252.212123642212</v>
       </c>
     </row>
     <row r="51">
@@ -12731,7 +13511,7 @@
       <c r="C51" s="3" t="n"/>
       <c r="D51" s="3" t="n"/>
       <c r="E51" s="4" t="n">
-        <v>3670.403875</v>
+        <v>3270.625336294613</v>
       </c>
     </row>
     <row r="52">
@@ -12748,7 +13528,7 @@
       <c r="C52" s="3" t="n"/>
       <c r="D52" s="3" t="n"/>
       <c r="E52" s="4" t="n">
-        <v>1512.55322</v>
+        <v>1511.12911517327</v>
       </c>
     </row>
   </sheetData>
@@ -12839,7 +13619,7 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>16.144040805</v>
+        <v>20.41556775550001</v>
       </c>
       <c r="D4" s="4" t="n">
         <v>20.4155677555</v>
@@ -12860,7 +13640,7 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>29.40549354</v>
+        <v>25.11669179</v>
       </c>
       <c r="D5" s="4" t="n">
         <v>25.11669179</v>
@@ -12902,7 +13682,7 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>0.9855513799999999</v>
+        <v>1.41922638</v>
       </c>
       <c r="D7" s="4" t="n">
         <v>1.41922638</v>
@@ -12923,7 +13703,7 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>114.14135412575</v>
+        <v>-33.99560463900924</v>
       </c>
       <c r="D8" s="4" t="n">
         <v>-33.9956046390092</v>
@@ -12944,7 +13724,7 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>688.1991265724987</v>
+        <v>718.1209297722988</v>
       </c>
       <c r="D9" s="4" t="n">
         <v>718.1209297723</v>
@@ -13007,7 +13787,7 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>2.0199435</v>
+        <v>2.04183504</v>
       </c>
       <c r="D12" s="4" t="n">
         <v>2.04183504</v>
@@ -13028,7 +13808,7 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>2.623159570000002</v>
+        <v>3.94193829</v>
       </c>
       <c r="D13" s="4" t="n">
         <v>3.94193829</v>
@@ -13091,7 +13871,7 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>0.3922464900000813</v>
+        <v>36.68221838000014</v>
       </c>
       <c r="D16" s="4" t="n">
         <v>36.68221838000012</v>
@@ -13112,7 +13892,7 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>103.78289826</v>
+        <v>110.3506010000001</v>
       </c>
       <c r="D17" s="4" t="n">
         <v>108.70517859</v>
@@ -13154,7 +13934,7 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>0.1337726</v>
+        <v>0</v>
       </c>
       <c r="D19" s="4" t="n">
         <v>0</v>
@@ -13175,7 +13955,7 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>17.09579156</v>
+        <v>12.9073848953064</v>
       </c>
       <c r="D20" s="4" t="n">
         <v>12.9073848953064</v>
@@ -13196,7 +13976,7 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>396.0007427899998</v>
+        <v>317.8970197199998</v>
       </c>
       <c r="D21" s="4" t="n">
         <v>317.89701972</v>
@@ -13217,7 +13997,7 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>0</v>
+        <v>35.08995146999995</v>
       </c>
       <c r="D22" s="4" t="n">
         <v>35.08995147</v>
@@ -13238,7 +14018,7 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>74.50949290999999</v>
+        <v>65.43014347000002</v>
       </c>
       <c r="D23" s="4" t="n">
         <v>65.43014347</v>
@@ -13259,7 +14039,7 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>281.1393901757846</v>
+        <v>289.4134120343151</v>
       </c>
       <c r="D24" s="4" t="n">
         <v>289.413412034315</v>
@@ -13280,7 +14060,7 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>2181.92665355782</v>
+        <v>1694.774720674792</v>
       </c>
       <c r="D25" s="4" t="n">
         <v>1694.774720674786</v>
@@ -13301,7 +14081,7 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>0</v>
+        <v>530.5244057082161</v>
       </c>
       <c r="D26" s="4" t="n">
         <v>530.524405708216</v>
@@ -13322,7 +14102,7 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>111.1991067368001</v>
+        <v>116.67142557</v>
       </c>
       <c r="D27" s="4" t="n">
         <v>116.67142557</v>
@@ -13343,7 +14123,7 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>49.01027474109002</v>
+        <v>33.82833946340012</v>
       </c>
       <c r="D28" s="4" t="n">
         <v>33.82833946340011</v>
@@ -13364,7 +14144,7 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>270.9919813645999</v>
+        <v>270.6326546714</v>
       </c>
       <c r="D29" s="4" t="n">
         <v>270.6326546714</v>
@@ -13427,7 +14207,7 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>5.941255356484301</v>
+        <v>2.883317708906</v>
       </c>
       <c r="D32" s="4" t="n">
         <v>2.883317708905999</v>
@@ -13448,7 +14228,7 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>138.35436699253</v>
+        <v>5.481413554157475</v>
       </c>
       <c r="D33" s="4" t="n">
         <v>5.481413554157481</v>
@@ -13490,7 +14270,7 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>13.08739285</v>
+        <v>20.55909881999998</v>
       </c>
       <c r="D35" s="4" t="n">
         <v>20.55909882</v>
@@ -13511,7 +14291,7 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>215.4481441199995</v>
+        <v>367.2996753195994</v>
       </c>
       <c r="D36" s="4" t="n">
         <v>367.2996753195995</v>
@@ -13532,7 +14312,7 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>2194.107870769827</v>
+        <v>2424.576406993308</v>
       </c>
       <c r="D37" s="4" t="n">
         <v>2424.576406993311</v>
@@ -13574,7 +14354,7 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>6.174234030549999</v>
+        <v>8.097845190549998</v>
       </c>
       <c r="D39" s="4" t="n">
         <v>8.09784519055</v>
@@ -13595,7 +14375,7 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>154.5083368053639</v>
+        <v>196.9777280472063</v>
       </c>
       <c r="D40" s="4" t="n">
         <v>196.9777280472059</v>
@@ -13616,7 +14396,7 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>2253.168970584798</v>
+        <v>1583.058037812898</v>
       </c>
       <c r="D41" s="4" t="n">
         <v>1583.0580378129</v>
@@ -13637,7 +14417,7 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>0</v>
+        <v>823.007257751496</v>
       </c>
       <c r="D42" s="4" t="n">
         <v>823.007257751496</v>
@@ -13713,7 +14493,7 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>1228.484651866455</v>
+        <v>1182.600091525276</v>
       </c>
       <c r="D3" s="4" t="n">
         <v>1182.600091525278</v>
@@ -13734,7 +14514,7 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>0</v>
+        <v>111.4715550414</v>
       </c>
       <c r="D4" s="4" t="n">
         <v>111.4715550414</v>
@@ -13755,7 +14535,7 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>0.6837</v>
+        <v>1.50242933</v>
       </c>
       <c r="D5" s="4" t="n">
         <v>1.50242933</v>
@@ -13776,7 +14556,7 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>4.79031256</v>
+        <v>4.74028056</v>
       </c>
       <c r="D6" s="4" t="n">
         <v>0</v>
@@ -13797,7 +14577,7 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>36.25447605</v>
+        <v>1651.14007755376</v>
       </c>
       <c r="D7" s="4" t="n">
         <v>1651.140077553759</v>
@@ -13818,7 +14598,7 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>3797.519876906318</v>
+        <v>3960.701672915284</v>
       </c>
       <c r="D8" s="4" t="n">
         <v>3960.701672915289</v>
@@ -13839,7 +14619,7 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>2960.087018881323</v>
+        <v>66.40347419613519</v>
       </c>
       <c r="D9" s="4" t="n">
         <v>66.40347419613519</v>
@@ -13860,7 +14640,7 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>108.6729605716756</v>
+        <v>0</v>
       </c>
       <c r="D10" s="4" t="n">
         <v>0</v>
@@ -13881,7 +14661,7 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>0</v>
+        <v>1388.621614929712</v>
       </c>
       <c r="D11" s="4" t="n">
         <v>1388.621614929712</v>
@@ -13902,7 +14682,7 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>95.67141705129988</v>
+        <v>63.4837640777999</v>
       </c>
       <c r="D12" s="4" t="n">
         <v>63.4837640777999</v>
@@ -13923,7 +14703,7 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>23.42895135</v>
+        <v>237.7633608235163</v>
       </c>
       <c r="D13" s="4" t="n">
         <v>237.7633608235163</v>
@@ -13944,7 +14724,7 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>4.220643740000003</v>
+        <v>7.101343170000005</v>
       </c>
       <c r="D14" s="4" t="n">
         <v>7.10134317</v>
@@ -13965,7 +14745,7 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>24.24665579679997</v>
+        <v>42.04669332891856</v>
       </c>
       <c r="D15" s="4" t="n">
         <v>42.04669332891851</v>
@@ -13986,7 +14766,7 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>82.93498648866115</v>
+        <v>86.38644855990059</v>
       </c>
       <c r="D16" s="4" t="n">
         <v>86.3864485599006</v>
@@ -14007,7 +14787,7 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>4.202896070000011</v>
+        <v>0.695049546999994</v>
       </c>
       <c r="D17" s="4" t="n">
         <v>0.695049546999996</v>
@@ -14028,7 +14808,7 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>143.5742110963009</v>
+        <v>-46.80343063892482</v>
       </c>
       <c r="D18" s="4" t="n">
         <v>-46.803430638925</v>
@@ -14049,7 +14829,7 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>0</v>
+        <v>311.0053714504</v>
       </c>
       <c r="D19" s="4" t="n">
         <v>311.0053714504</v>
@@ -14070,7 +14850,7 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>84.54519621919999</v>
+        <v>107.53940529857</v>
       </c>
       <c r="D20" s="4" t="n">
         <v>107.53940529857</v>
@@ -14091,7 +14871,7 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>25.75025801796</v>
+        <v>53.40910758</v>
       </c>
       <c r="D21" s="4" t="n">
         <v>53.40910758</v>
@@ -14112,7 +14892,7 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>453.1498506605509</v>
+        <v>237.7633608235163</v>
       </c>
       <c r="D22" s="4" t="n">
         <v>0</v>
@@ -14133,7 +14913,7 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>206.51471250735</v>
+        <v>189.9621334005501</v>
       </c>
       <c r="D23" s="4" t="n">
         <v>189.96213340055</v>
@@ -14154,7 +14934,7 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>60.36629896111748</v>
+        <v>263.8583619950439</v>
       </c>
       <c r="D24" s="4" t="n">
         <v>266.9532201450451</v>
@@ -14219,7 +14999,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>837.2622501330402</v>
+        <v>261.0126084473399</v>
       </c>
       <c r="C3" s="4" t="n">
         <v>261.01260844734</v>
@@ -14235,7 +15015,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>840.9156452053561</v>
+        <v>429.9093362272502</v>
       </c>
       <c r="C4" s="4" t="n">
         <v>429.90933622725</v>
@@ -14251,7 +15031,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>317.7136080464301</v>
+        <v>185.1237281950259</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>185.123728195026</v>
@@ -14267,7 +15047,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>379.5619179905914</v>
+        <v>828.8096792800516</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>828.809679280051</v>
@@ -14283,7 +15063,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>339.0399439599998</v>
+        <v>351.3839240000001</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>351.383924</v>
@@ -14299,7 +15079,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>676.8623477589564</v>
+        <v>565.5785141719452</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>565.578514171944</v>
@@ -14428,7 +15208,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>16.36384947937154</v>
+        <v>15.34698462943654</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>15.3469846294365</v>
@@ -14444,7 +15224,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>65.07301663641621</v>
+        <v>67.29213861641628</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>67.29213861641631</v>
@@ -14460,7 +15240,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>228.1029684089168</v>
+        <v>276.1146507064188</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>276.114650706419</v>
@@ -14476,7 +15256,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>5225.334241604624</v>
+        <v>4211.70881054095</v>
       </c>
       <c r="C10" s="4" t="n">
         <v>4211.70881054095</v>
@@ -14492,7 +15272,7 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>7699.535192548273</v>
+        <v>8277.110015976186</v>
       </c>
       <c r="C11" s="4" t="n">
         <v>8275.46459356617</v>
@@ -14508,7 +15288,7 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>2.182787284255028e-11</v>
+        <v>0</v>
       </c>
       <c r="C12" s="4" t="n">
         <v>4.001776687800884e-11</v>

</xml_diff>